<commit_message>
docs: étendre le fichier d'import d'exemple aux 6 départements
</commit_message>
<xml_diff>
--- a/docs/exemples/liste-blanche-exemple.xlsx
+++ b/docs/exemples/liste-blanche-exemple.xlsx
@@ -12,7 +12,7 @@
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -103,12 +103,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>DUT1</t>
+          <t>DUT2</t>
         </is>
       </c>
     </row>
@@ -140,7 +140,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>DUT1</t>
+          <t>DIC1</t>
         </is>
       </c>
     </row>
@@ -172,7 +172,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>DUT2</t>
+          <t>DIC2</t>
         </is>
       </c>
     </row>
@@ -199,12 +199,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DUT2</t>
+          <t>DIC3</t>
         </is>
       </c>
     </row>
@@ -226,17 +226,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Mécanique</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DUT2</t>
+          <t>DUT1</t>
         </is>
       </c>
     </row>
@@ -258,17 +258,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Mécanique</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>DIC1</t>
+          <t>DUT2</t>
         </is>
       </c>
     </row>
@@ -290,7 +290,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Mécanique</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -322,7 +322,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Mécanique</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -354,17 +354,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Mécanique</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DIC2</t>
+          <t>DIC3</t>
         </is>
       </c>
     </row>
@@ -386,17 +386,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Chimique et Biologie Appliquée</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>DIC3</t>
+          <t>DUT1</t>
         </is>
       </c>
     </row>
@@ -418,15 +418,591 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Génie Informatique</t>
+          <t>Génie Chimique et Biologie Appliquée</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DUT2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cissé</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Aïssatou</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>exemple.aissatou.cisse@esp.sn</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Génie Chimique et Biologie Appliquée</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>DIC1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mbaye</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Babacar</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>exemple.babacar.mbaye@esp.sn</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Génie Chimique et Biologie Appliquée</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>DIC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sy</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Coumba</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>exemple.coumba.sy@gmail.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Génie Chimique et Biologie Appliquée</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>DIC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Dieng</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Modou</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>exemple.modou.dieng@esp.sn</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Génie Électrique</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>DUT1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Lô</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Rokhaya</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>exemple.rokhaya.lo@esp.sn</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Génie Électrique</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>DUT2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Camara</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Pape</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>exemple.pape.camara@gmail.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Génie Électrique</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>DIC1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Touré</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sokhna</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>exemple.sokhna.toure@esp.sn</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Génie Électrique</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>DIC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Badji</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Alioune</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>exemple.alioune.badji@esp.sn</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Génie Électrique</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>DIC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Niang</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bineta</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>exemple.bineta.niang@gmail.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Génie Civil</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>DUT1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wade</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Serigne</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>exemple.serigne.wade@esp.sn</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Génie Civil</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>DUT2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Samb</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dieynaba</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>exemple.dieynaba.samb@esp.sn</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Génie Civil</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>DIC1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Dia</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lamine</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>exemple.lamine.dia@gmail.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Génie Civil</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DIC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mendy</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Astou</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>exemple.astou.mendy@esp.sn</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Génie Civil</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>DIC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tall</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Malick</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>exemple.malick.tall@esp.sn</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>DUT1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ndour</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Oumou</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>exemple.oumou.ndour@gmail.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>DUT2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Diouf</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Souleymane</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>exemple.souleymane.diouf@esp.sn</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>DIC1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sène</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Yacine</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>exemple.yacine.sene@esp.sn</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>DIC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Guèye</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>El Hadji</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>exemple.elhadji.gueye@gmail.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>DIC3</t>
         </is>

</xml_diff>